<commit_message>
Generate editable spreadsheet with database schema and data
Co-authored-by: michieltw <300185964+michieltw@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Spreadsheet_editable.xlsx
+++ b/Spreadsheet_editable.xlsx
@@ -18933,7 +18933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19182,7 +19182,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_0__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -19196,7 +19196,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_3__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -19210,7 +19210,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_6__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -19224,7 +19224,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_9__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -19238,77 +19238,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_12__</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
           <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_15__</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_18__</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_21__</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_24__</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>SELECT id FROM arenas WHERE name = __STR_27__</t>
         </is>
       </c>
     </row>
@@ -60474,7 +60404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60713,7 +60643,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_0__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -60727,7 +60657,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_3__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -60741,7 +60671,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_6__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -60755,7 +60685,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_9__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -60769,77 +60699,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_12__</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
           <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_15__</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_18__</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_21__</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_24__</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_27__</t>
         </is>
       </c>
     </row>
@@ -67175,7 +67035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67348,7 +67208,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_0__</t>
+          <t>gen_random_uuid(</t>
         </is>
       </c>
     </row>
@@ -67362,35 +67222,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_1__</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
           <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_2__</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>gen_random_uuid(</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>SELECT id FROM organizations WHERE name = __STR_3__</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Benelux ice hockey data to spreadsheet
- Appended new rows for Benelux-specific arenas, clubs, leagues, and
  organizations (e.g., Tilburg Trappers, Hijs Hokij Den Haag,
  Liege Bulldogs, CEHL, Eredivisie) to Spreadsheet_editable.xlsx.
- Formatted all newly added rows with a yellow background (FFFF00).

Co-authored-by: michieltw <300185964+michieltw@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Spreadsheet_editable.xlsx
+++ b/Spreadsheet_editable.xlsx
@@ -911,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1515,6 +1515,201 @@
       <c r="U8" s="1" t="n"/>
       <c r="V8" s="1" t="n"/>
       <c r="W8" s="1" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="1" t="n"/>
+      <c r="D9" s="1" t="n"/>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>'Central European Hockey League'</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>'CEHL'</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>'Semi-Professional'</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>'Men'</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="n"/>
+      <c r="L9" s="1" t="n"/>
+      <c r="M9" s="1" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="N9" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.cehl.eu'</t>
+        </is>
+      </c>
+      <c r="O9" s="1" t="n"/>
+      <c r="P9" s="1" t="n"/>
+      <c r="Q9" s="1" t="n"/>
+      <c r="R9" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S9" s="1" t="n"/>
+      <c r="T9" s="1" t="n"/>
+      <c r="U9" s="1" t="n"/>
+      <c r="V9" s="1" t="n"/>
+      <c r="W9" s="1" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>'Eredivisie'</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>'Amateur'</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="inlineStr">
+        <is>
+          <t>'Men'</t>
+        </is>
+      </c>
+      <c r="K10" s="1" t="n"/>
+      <c r="L10" s="1" t="n"/>
+      <c r="M10" s="1" t="inlineStr">
+        <is>
+          <t>1945</t>
+        </is>
+      </c>
+      <c r="N10" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.ijshockeynederland.nl'</t>
+        </is>
+      </c>
+      <c r="O10" s="1" t="n"/>
+      <c r="P10" s="1" t="n"/>
+      <c r="Q10" s="1" t="n"/>
+      <c r="R10" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S10" s="1" t="n"/>
+      <c r="T10" s="1" t="n"/>
+      <c r="U10" s="1" t="n"/>
+      <c r="V10" s="1" t="n"/>
+      <c r="W10" s="1" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Royal Belgian Ice Hockey Federation')</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>'Belgian National League'</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>'Amateur'</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J11" s="1" t="inlineStr">
+        <is>
+          <t>'Men'</t>
+        </is>
+      </c>
+      <c r="K11" s="1" t="n"/>
+      <c r="L11" s="1" t="n"/>
+      <c r="M11" s="1" t="inlineStr">
+        <is>
+          <t>1912</t>
+        </is>
+      </c>
+      <c r="N11" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.rbihf.be'</t>
+        </is>
+      </c>
+      <c r="O11" s="1" t="n"/>
+      <c r="P11" s="1" t="n"/>
+      <c r="Q11" s="1" t="n"/>
+      <c r="R11" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S11" s="1" t="n"/>
+      <c r="T11" s="1" t="n"/>
+      <c r="U11" s="1" t="n"/>
+      <c r="V11" s="1" t="n"/>
+      <c r="W11" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9124,7 +9319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T32"/>
+  <dimension ref="A1:T42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10575,6 +10770,566 @@
       <c r="R32" s="1" t="n"/>
       <c r="S32" s="1" t="n"/>
       <c r="T32" s="1" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>'Tilburg Trappers'</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>'TIL'</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>1938</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.trappers.nl'</t>
+        </is>
+      </c>
+      <c r="H33" s="1" t="n"/>
+      <c r="I33" s="1" t="n"/>
+      <c r="J33" s="1" t="n"/>
+      <c r="K33" s="1" t="n"/>
+      <c r="L33" s="1" t="n"/>
+      <c r="M33" s="1" t="inlineStr">
+        <is>
+          <t>'Tilburg'</t>
+        </is>
+      </c>
+      <c r="N33" s="1" t="n"/>
+      <c r="O33" s="1" t="n"/>
+      <c r="P33" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q33" s="1" t="inlineStr">
+        <is>
+          <t>'Professional Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R33" s="1" t="n"/>
+      <c r="S33" s="1" t="n"/>
+      <c r="T33" s="1" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="n"/>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>'Hijs Hokij Den Haag'</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>'DEN'</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>1933</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.hijshokij.nl'</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="n"/>
+      <c r="I34" s="1" t="n"/>
+      <c r="J34" s="1" t="n"/>
+      <c r="K34" s="1" t="n"/>
+      <c r="L34" s="1" t="n"/>
+      <c r="M34" s="1" t="inlineStr">
+        <is>
+          <t>'The Hague'</t>
+        </is>
+      </c>
+      <c r="N34" s="1" t="n"/>
+      <c r="O34" s="1" t="n"/>
+      <c r="P34" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q34" s="1" t="inlineStr">
+        <is>
+          <t>'CEHL Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R34" s="1" t="n"/>
+      <c r="S34" s="1" t="n"/>
+      <c r="T34" s="1" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="n"/>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>'UNIS Flyers Heerenveen'</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>'HEE'</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>1967</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.unisflyers.nl'</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="n"/>
+      <c r="I35" s="1" t="n"/>
+      <c r="J35" s="1" t="n"/>
+      <c r="K35" s="1" t="n"/>
+      <c r="L35" s="1" t="n"/>
+      <c r="M35" s="1" t="inlineStr">
+        <is>
+          <t>'Heerenveen'</t>
+        </is>
+      </c>
+      <c r="N35" s="1" t="n"/>
+      <c r="O35" s="1" t="n"/>
+      <c r="P35" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q35" s="1" t="inlineStr">
+        <is>
+          <t>'CEHL Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R35" s="1" t="n"/>
+      <c r="S35" s="1" t="n"/>
+      <c r="T35" s="1" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>'Snackpoint Eaters Limburg'</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>'EAT'</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>1968</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.eaters.nl'</t>
+        </is>
+      </c>
+      <c r="H36" s="1" t="n"/>
+      <c r="I36" s="1" t="n"/>
+      <c r="J36" s="1" t="n"/>
+      <c r="K36" s="1" t="n"/>
+      <c r="L36" s="1" t="n"/>
+      <c r="M36" s="1" t="inlineStr">
+        <is>
+          <t>'Geleen'</t>
+        </is>
+      </c>
+      <c r="N36" s="1" t="n"/>
+      <c r="O36" s="1" t="n"/>
+      <c r="P36" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q36" s="1" t="inlineStr">
+        <is>
+          <t>'CEHL Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R36" s="1" t="n"/>
+      <c r="S36" s="1" t="n"/>
+      <c r="T36" s="1" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>'Liege Bulldogs'</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>'LIE'</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.bulldogs-liege.be'</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="n"/>
+      <c r="I37" s="1" t="n"/>
+      <c r="J37" s="1" t="n"/>
+      <c r="K37" s="1" t="n"/>
+      <c r="L37" s="1" t="n"/>
+      <c r="M37" s="1" t="inlineStr">
+        <is>
+          <t>'Liège'</t>
+        </is>
+      </c>
+      <c r="N37" s="1" t="n"/>
+      <c r="O37" s="1" t="n"/>
+      <c r="P37" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="Q37" s="1" t="inlineStr">
+        <is>
+          <t>'CEHL Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R37" s="1" t="n"/>
+      <c r="S37" s="1" t="n"/>
+      <c r="T37" s="1" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="n"/>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>'HYC Herentals'</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>'HYC'</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>1971</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.hyc.be'</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="n"/>
+      <c r="I38" s="1" t="n"/>
+      <c r="J38" s="1" t="n"/>
+      <c r="K38" s="1" t="n"/>
+      <c r="L38" s="1" t="n"/>
+      <c r="M38" s="1" t="inlineStr">
+        <is>
+          <t>'Herentals'</t>
+        </is>
+      </c>
+      <c r="N38" s="1" t="n"/>
+      <c r="O38" s="1" t="n"/>
+      <c r="P38" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="Q38" s="1" t="inlineStr">
+        <is>
+          <t>'CEHL Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R38" s="1" t="n"/>
+      <c r="S38" s="1" t="n"/>
+      <c r="T38" s="1" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="n"/>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>'Tornado Luxembourg'</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>'TOR'</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>1987</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.tornadoluxembourg.com'</t>
+        </is>
+      </c>
+      <c r="H39" s="1" t="n"/>
+      <c r="I39" s="1" t="n"/>
+      <c r="J39" s="1" t="n"/>
+      <c r="K39" s="1" t="n"/>
+      <c r="L39" s="1" t="n"/>
+      <c r="M39" s="1" t="inlineStr">
+        <is>
+          <t>'Luxembourg City'</t>
+        </is>
+      </c>
+      <c r="N39" s="1" t="n"/>
+      <c r="O39" s="1" t="n"/>
+      <c r="P39" s="1" t="inlineStr">
+        <is>
+          <t>'Luxembourg'</t>
+        </is>
+      </c>
+      <c r="Q39" s="1" t="inlineStr">
+        <is>
+          <t>'Ice Hockey Team in Luxembourg'</t>
+        </is>
+      </c>
+      <c r="R39" s="1" t="n"/>
+      <c r="S39" s="1" t="n"/>
+      <c r="T39" s="1" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="n"/>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>'League'</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>'Central European Hockey League'</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>'CEHL'</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.cehl.eu'</t>
+        </is>
+      </c>
+      <c r="H40" s="1" t="n"/>
+      <c r="I40" s="1" t="n"/>
+      <c r="J40" s="1" t="n"/>
+      <c r="K40" s="1" t="n"/>
+      <c r="L40" s="1" t="n"/>
+      <c r="M40" s="1" t="n"/>
+      <c r="N40" s="1" t="n"/>
+      <c r="O40" s="1" t="n"/>
+      <c r="P40" s="1" t="inlineStr">
+        <is>
+          <t>'Europe'</t>
+        </is>
+      </c>
+      <c r="Q40" s="1" t="inlineStr">
+        <is>
+          <t>'Top level ice hockey league in the Benelux'</t>
+        </is>
+      </c>
+      <c r="R40" s="1" t="n"/>
+      <c r="S40" s="1" t="n"/>
+      <c r="T40" s="1" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="n"/>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>'League'</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>'Eredivisie'</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="n"/>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>1945</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.ijshockeynederland.nl'</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="n"/>
+      <c r="I41" s="1" t="n"/>
+      <c r="J41" s="1" t="n"/>
+      <c r="K41" s="1" t="n"/>
+      <c r="L41" s="1" t="n"/>
+      <c r="M41" s="1" t="n"/>
+      <c r="N41" s="1" t="n"/>
+      <c r="O41" s="1" t="n"/>
+      <c r="P41" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q41" s="1" t="inlineStr">
+        <is>
+          <t>'Dutch national ice hockey league'</t>
+        </is>
+      </c>
+      <c r="R41" s="1" t="n"/>
+      <c r="S41" s="1" t="n"/>
+      <c r="T41" s="1" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="n"/>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>'League'</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>'Belgian National League'</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="n"/>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>1912</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.rbihf.be'</t>
+        </is>
+      </c>
+      <c r="H42" s="1" t="n"/>
+      <c r="I42" s="1" t="n"/>
+      <c r="J42" s="1" t="n"/>
+      <c r="K42" s="1" t="n"/>
+      <c r="L42" s="1" t="n"/>
+      <c r="M42" s="1" t="n"/>
+      <c r="N42" s="1" t="n"/>
+      <c r="O42" s="1" t="n"/>
+      <c r="P42" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="Q42" s="1" t="inlineStr">
+        <is>
+          <t>'Belgian national ice hockey league'</t>
+        </is>
+      </c>
+      <c r="R42" s="1" t="n"/>
+      <c r="S42" s="1" t="n"/>
+      <c r="T42" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16651,7 +17406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18231,6 +18986,300 @@
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="n"/>
       <c r="Q47" s="1" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="n"/>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>'IJssportcentrum Stappegoor'</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="n"/>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>'Stappegoorweg 3'</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>'Tilburg'</t>
+        </is>
+      </c>
+      <c r="I48" s="1" t="n"/>
+      <c r="J48" s="1" t="inlineStr">
+        <is>
+          <t>'5022 DA'</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L48" s="1" t="n"/>
+      <c r="M48" s="1" t="n"/>
+      <c r="N48" s="1" t="n"/>
+      <c r="O48" s="1" t="n"/>
+      <c r="P48" s="1" t="n"/>
+      <c r="Q48" s="1" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="n"/>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>'De Uithof'</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="n"/>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>2610</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>'Jaap Edenweg 10'</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>'The Hague'</t>
+        </is>
+      </c>
+      <c r="I49" s="1" t="n"/>
+      <c r="J49" s="1" t="inlineStr">
+        <is>
+          <t>'2544 NL'</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L49" s="1" t="n"/>
+      <c r="M49" s="1" t="n"/>
+      <c r="N49" s="1" t="n"/>
+      <c r="O49" s="1" t="n"/>
+      <c r="P49" s="1" t="n"/>
+      <c r="Q49" s="1" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="n"/>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>'Glanerbrook'</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="n"/>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="n"/>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>'Kummenaedestraat 45'</t>
+        </is>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>'Geleen'</t>
+        </is>
+      </c>
+      <c r="I50" s="1" t="n"/>
+      <c r="J50" s="1" t="inlineStr">
+        <is>
+          <t>'6165 BT'</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L50" s="1" t="n"/>
+      <c r="M50" s="1" t="n"/>
+      <c r="N50" s="1" t="n"/>
+      <c r="O50" s="1" t="n"/>
+      <c r="P50" s="1" t="n"/>
+      <c r="Q50" s="1" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="n"/>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>'Patinoire de Liège'</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="n"/>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>1250</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>'Boulevard Raymond Poincaré 7'</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>'Liège'</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="n"/>
+      <c r="J51" s="1" t="inlineStr">
+        <is>
+          <t>'4020'</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="L51" s="1" t="n"/>
+      <c r="M51" s="1" t="n"/>
+      <c r="N51" s="1" t="n"/>
+      <c r="O51" s="1" t="n"/>
+      <c r="P51" s="1" t="n"/>
+      <c r="Q51" s="1" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="n"/>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>'Bloso Centrum Netepark'</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="n"/>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="n"/>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>'Vorselaarsebaan 60'</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>'Herentals'</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="n"/>
+      <c r="J52" s="1" t="inlineStr">
+        <is>
+          <t>'2200'</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="L52" s="1" t="n"/>
+      <c r="M52" s="1" t="n"/>
+      <c r="N52" s="1" t="n"/>
+      <c r="O52" s="1" t="n"/>
+      <c r="P52" s="1" t="n"/>
+      <c r="Q52" s="1" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="n"/>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>'Patinoire de Kockelscheuer'</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="n"/>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="n"/>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>'Route de Bettembourg 42'</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>'Kockelscheuer'</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="n"/>
+      <c r="J53" s="1" t="inlineStr">
+        <is>
+          <t>'1899'</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>'Luxembourg'</t>
+        </is>
+      </c>
+      <c r="L53" s="1" t="n"/>
+      <c r="M53" s="1" t="n"/>
+      <c r="N53" s="1" t="n"/>
+      <c r="O53" s="1" t="n"/>
+      <c r="P53" s="1" t="n"/>
+      <c r="Q53" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -59510,7 +60559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60058,6 +61107,272 @@
       <c r="J18" s="1" t="n"/>
       <c r="K18" s="1" t="n"/>
       <c r="L18" s="1" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="n"/>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Tilburg Trappers')</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'IJssportcentrum Stappegoor')</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>'#00448A'</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>'#FFC82E'</t>
+        </is>
+      </c>
+      <c r="H19" s="1" t="n"/>
+      <c r="I19" s="1" t="n"/>
+      <c r="J19" s="1" t="n"/>
+      <c r="K19" s="1" t="n"/>
+      <c r="L19" s="1" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Hijs Hokij Den Haag')</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'De Uithof')</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>'#E2001A'</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>'#000000'</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="n"/>
+      <c r="I20" s="1" t="n"/>
+      <c r="J20" s="1" t="n"/>
+      <c r="K20" s="1" t="n"/>
+      <c r="L20" s="1" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="n"/>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'UNIS Flyers Heerenveen')</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Thialf Ice Stadium')</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>'#D50032'</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H21" s="1" t="n"/>
+      <c r="I21" s="1" t="n"/>
+      <c r="J21" s="1" t="n"/>
+      <c r="K21" s="1" t="n"/>
+      <c r="L21" s="1" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="n"/>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Snackpoint Eaters Limburg')</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Glanerbrook')</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>'#C8102E'</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>'#000000'</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="n"/>
+      <c r="I22" s="1" t="n"/>
+      <c r="J22" s="1" t="n"/>
+      <c r="K22" s="1" t="n"/>
+      <c r="L22" s="1" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="n"/>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Liege Bulldogs')</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Royal Belgian Ice Hockey Federation')</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Patinoire de Liège')</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>'#0055A4'</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>'#EF4135'</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="n"/>
+      <c r="I23" s="1" t="n"/>
+      <c r="J23" s="1" t="n"/>
+      <c r="K23" s="1" t="n"/>
+      <c r="L23" s="1" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="n"/>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'HYC Herentals')</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Royal Belgian Ice Hockey Federation')</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Bloso Centrum Netepark')</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>'#E30613'</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="n"/>
+      <c r="I24" s="1" t="n"/>
+      <c r="J24" s="1" t="n"/>
+      <c r="K24" s="1" t="n"/>
+      <c r="L24" s="1" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="n"/>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Tornado Luxembourg')</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Fédération Luxembourgeoise de Hockey sur Glace')</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Patinoire de Kockelscheuer')</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>'#002C5F'</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>'#F37021'</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="n"/>
+      <c r="I25" s="1" t="n"/>
+      <c r="J25" s="1" t="n"/>
+      <c r="K25" s="1" t="n"/>
+      <c r="L25" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add lower-level Benelux teams and upcoming season to spreadsheet
- Appended new rows for Eerste Divisie and Belgian National League
  Division 2 teams (e.g., Amsterdam Tigers, GIJS Groningen, Nijmegen
  Devils, IHC Leuven, Phantoms Antwerp).
- Added corresponding arenas to the 'arenas' sheet.
- Added '2024-2025' to the 'seasons' sheet.
- Formatted all newly added rows with a yellow background (FFFF00).

Co-authored-by: michieltw <300185964+michieltw@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Spreadsheet_editable.xlsx
+++ b/Spreadsheet_editable.xlsx
@@ -911,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1710,6 +1710,136 @@
       <c r="U11" s="1" t="n"/>
       <c r="V11" s="1" t="n"/>
       <c r="W11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie'</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>'Amateur'</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>'Men'</t>
+        </is>
+      </c>
+      <c r="K12" s="1" t="n"/>
+      <c r="L12" s="1" t="n"/>
+      <c r="M12" s="1" t="inlineStr">
+        <is>
+          <t>1945</t>
+        </is>
+      </c>
+      <c r="N12" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.ijshockeynederland.nl'</t>
+        </is>
+      </c>
+      <c r="O12" s="1" t="n"/>
+      <c r="P12" s="1" t="n"/>
+      <c r="Q12" s="1" t="n"/>
+      <c r="R12" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S12" s="1" t="n"/>
+      <c r="T12" s="1" t="n"/>
+      <c r="U12" s="1" t="n"/>
+      <c r="V12" s="1" t="n"/>
+      <c r="W12" s="1" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Royal Belgian Ice Hockey Federation')</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="n"/>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>'Belgian National League Division 2'</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="n"/>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>'Amateur'</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr">
+        <is>
+          <t>'Men'</t>
+        </is>
+      </c>
+      <c r="K13" s="1" t="n"/>
+      <c r="L13" s="1" t="n"/>
+      <c r="M13" s="1" t="inlineStr">
+        <is>
+          <t>1912</t>
+        </is>
+      </c>
+      <c r="N13" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.rbihf.be'</t>
+        </is>
+      </c>
+      <c r="O13" s="1" t="n"/>
+      <c r="P13" s="1" t="n"/>
+      <c r="Q13" s="1" t="n"/>
+      <c r="R13" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S13" s="1" t="n"/>
+      <c r="T13" s="1" t="n"/>
+      <c r="U13" s="1" t="n"/>
+      <c r="V13" s="1" t="n"/>
+      <c r="W13" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9319,7 +9449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T42"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11330,6 +11460,802 @@
       <c r="R42" s="1" t="n"/>
       <c r="S42" s="1" t="n"/>
       <c r="T42" s="1" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="n"/>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>'Amsterdam Tigers'</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>'AMS'</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>1963</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.amsterdamtigers.com'</t>
+        </is>
+      </c>
+      <c r="H43" s="1" t="n"/>
+      <c r="I43" s="1" t="n"/>
+      <c r="J43" s="1" t="n"/>
+      <c r="K43" s="1" t="n"/>
+      <c r="L43" s="1" t="n"/>
+      <c r="M43" s="1" t="inlineStr">
+        <is>
+          <t>'Amsterdam'</t>
+        </is>
+      </c>
+      <c r="N43" s="1" t="n"/>
+      <c r="O43" s="1" t="n"/>
+      <c r="P43" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q43" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R43" s="1" t="n"/>
+      <c r="S43" s="1" t="n"/>
+      <c r="T43" s="1" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="n"/>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>'GIJS Groningen'</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>'GRO'</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>1969</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.gijsgroningen.nl'</t>
+        </is>
+      </c>
+      <c r="H44" s="1" t="n"/>
+      <c r="I44" s="1" t="n"/>
+      <c r="J44" s="1" t="n"/>
+      <c r="K44" s="1" t="n"/>
+      <c r="L44" s="1" t="n"/>
+      <c r="M44" s="1" t="inlineStr">
+        <is>
+          <t>'Groningen'</t>
+        </is>
+      </c>
+      <c r="N44" s="1" t="n"/>
+      <c r="O44" s="1" t="n"/>
+      <c r="P44" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q44" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R44" s="1" t="n"/>
+      <c r="S44" s="1" t="n"/>
+      <c r="T44" s="1" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="n"/>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>'Nijmegen Devils'</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>'NIJ'</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>1969</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.nijmegendevils.nl'</t>
+        </is>
+      </c>
+      <c r="H45" s="1" t="n"/>
+      <c r="I45" s="1" t="n"/>
+      <c r="J45" s="1" t="n"/>
+      <c r="K45" s="1" t="n"/>
+      <c r="L45" s="1" t="n"/>
+      <c r="M45" s="1" t="inlineStr">
+        <is>
+          <t>'Nijmegen'</t>
+        </is>
+      </c>
+      <c r="N45" s="1" t="n"/>
+      <c r="O45" s="1" t="n"/>
+      <c r="P45" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q45" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R45" s="1" t="n"/>
+      <c r="S45" s="1" t="n"/>
+      <c r="T45" s="1" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="n"/>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>'Red Eagles ''s-Hertogenbosch'</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>'RED'</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.redeagles.nl'</t>
+        </is>
+      </c>
+      <c r="H46" s="1" t="n"/>
+      <c r="I46" s="1" t="n"/>
+      <c r="J46" s="1" t="n"/>
+      <c r="K46" s="1" t="n"/>
+      <c r="L46" s="1" t="n"/>
+      <c r="M46" s="1" t="inlineStr">
+        <is>
+          <t>'s-Hertogenbosch'</t>
+        </is>
+      </c>
+      <c r="N46" s="1" t="n"/>
+      <c r="O46" s="1" t="n"/>
+      <c r="P46" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q46" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R46" s="1" t="n"/>
+      <c r="S46" s="1" t="n"/>
+      <c r="T46" s="1" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="n"/>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>'Yeti''s Breda'</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>'YET'</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.yetisbreda.nl'</t>
+        </is>
+      </c>
+      <c r="H47" s="1" t="n"/>
+      <c r="I47" s="1" t="n"/>
+      <c r="J47" s="1" t="n"/>
+      <c r="K47" s="1" t="n"/>
+      <c r="L47" s="1" t="n"/>
+      <c r="M47" s="1" t="inlineStr">
+        <is>
+          <t>'Breda'</t>
+        </is>
+      </c>
+      <c r="N47" s="1" t="n"/>
+      <c r="O47" s="1" t="n"/>
+      <c r="P47" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q47" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R47" s="1" t="n"/>
+      <c r="S47" s="1" t="n"/>
+      <c r="T47" s="1" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="n"/>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>'Zoetermeer Panters'</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>'ZOE'</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>1979</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.panters.nl'</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="n"/>
+      <c r="I48" s="1" t="n"/>
+      <c r="J48" s="1" t="n"/>
+      <c r="K48" s="1" t="n"/>
+      <c r="L48" s="1" t="n"/>
+      <c r="M48" s="1" t="inlineStr">
+        <is>
+          <t>'Zoetermeer'</t>
+        </is>
+      </c>
+      <c r="N48" s="1" t="n"/>
+      <c r="O48" s="1" t="n"/>
+      <c r="P48" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q48" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R48" s="1" t="n"/>
+      <c r="S48" s="1" t="n"/>
+      <c r="T48" s="1" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="n"/>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>'IHC Leuven'</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>'LEU'</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.ihcleuven.be'</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="n"/>
+      <c r="I49" s="1" t="n"/>
+      <c r="J49" s="1" t="n"/>
+      <c r="K49" s="1" t="n"/>
+      <c r="L49" s="1" t="n"/>
+      <c r="M49" s="1" t="inlineStr">
+        <is>
+          <t>'Leuven'</t>
+        </is>
+      </c>
+      <c r="N49" s="1" t="n"/>
+      <c r="O49" s="1" t="n"/>
+      <c r="P49" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="Q49" s="1" t="inlineStr">
+        <is>
+          <t>'Belgian National League Team'</t>
+        </is>
+      </c>
+      <c r="R49" s="1" t="n"/>
+      <c r="S49" s="1" t="n"/>
+      <c r="T49" s="1" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="n"/>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>'Phantoms Antwerp'</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>'PHA'</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.phantoms.be'</t>
+        </is>
+      </c>
+      <c r="H50" s="1" t="n"/>
+      <c r="I50" s="1" t="n"/>
+      <c r="J50" s="1" t="n"/>
+      <c r="K50" s="1" t="n"/>
+      <c r="L50" s="1" t="n"/>
+      <c r="M50" s="1" t="inlineStr">
+        <is>
+          <t>'Antwerp'</t>
+        </is>
+      </c>
+      <c r="N50" s="1" t="n"/>
+      <c r="O50" s="1" t="n"/>
+      <c r="P50" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="Q50" s="1" t="inlineStr">
+        <is>
+          <t>'Belgian National League Team'</t>
+        </is>
+      </c>
+      <c r="R50" s="1" t="n"/>
+      <c r="S50" s="1" t="n"/>
+      <c r="T50" s="1" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="n"/>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>'League'</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie'</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="n"/>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>1945</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.ijshockeynederland.nl'</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="n"/>
+      <c r="I51" s="1" t="n"/>
+      <c r="J51" s="1" t="n"/>
+      <c r="K51" s="1" t="n"/>
+      <c r="L51" s="1" t="n"/>
+      <c r="M51" s="1" t="n"/>
+      <c r="N51" s="1" t="n"/>
+      <c r="O51" s="1" t="n"/>
+      <c r="P51" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q51" s="1" t="inlineStr">
+        <is>
+          <t>'Dutch second-tier ice hockey league'</t>
+        </is>
+      </c>
+      <c r="R51" s="1" t="n"/>
+      <c r="S51" s="1" t="n"/>
+      <c r="T51" s="1" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="n"/>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>'League'</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>'Belgian National League Division 2'</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="n"/>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>1912</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.rbihf.be'</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="n"/>
+      <c r="I52" s="1" t="n"/>
+      <c r="J52" s="1" t="n"/>
+      <c r="K52" s="1" t="n"/>
+      <c r="L52" s="1" t="n"/>
+      <c r="M52" s="1" t="n"/>
+      <c r="N52" s="1" t="n"/>
+      <c r="O52" s="1" t="n"/>
+      <c r="P52" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="Q52" s="1" t="inlineStr">
+        <is>
+          <t>'Belgian second-tier ice hockey league'</t>
+        </is>
+      </c>
+      <c r="R52" s="1" t="n"/>
+      <c r="S52" s="1" t="n"/>
+      <c r="T52" s="1" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="n"/>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>'Leeuwarden Warriors'</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>'LEU'</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.ijshockeyleeuwarden.nl/'</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="n"/>
+      <c r="I53" s="1" t="n"/>
+      <c r="J53" s="1" t="n"/>
+      <c r="K53" s="1" t="n"/>
+      <c r="L53" s="1" t="n"/>
+      <c r="M53" s="1" t="inlineStr">
+        <is>
+          <t>'Leeuwarden'</t>
+        </is>
+      </c>
+      <c r="N53" s="1" t="n"/>
+      <c r="O53" s="1" t="n"/>
+      <c r="P53" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q53" s="1" t="inlineStr">
+        <is>
+          <t>'Eerste Divisie Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R53" s="1" t="n"/>
+      <c r="S53" s="1" t="n"/>
+      <c r="T53" s="1" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="n"/>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>'Alcmaria Flames'</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>'ALC'</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>1971</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.alcmariaflames.nl/'</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="n"/>
+      <c r="I54" s="1" t="n"/>
+      <c r="J54" s="1" t="n"/>
+      <c r="K54" s="1" t="n"/>
+      <c r="L54" s="1" t="n"/>
+      <c r="M54" s="1" t="inlineStr">
+        <is>
+          <t>'Alkmaar'</t>
+        </is>
+      </c>
+      <c r="N54" s="1" t="n"/>
+      <c r="O54" s="1" t="n"/>
+      <c r="P54" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q54" s="1" t="inlineStr">
+        <is>
+          <t>'Dutch Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R54" s="1" t="n"/>
+      <c r="S54" s="1" t="n"/>
+      <c r="T54" s="1" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="n"/>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>'Dordrecht Lions'</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>'DOR'</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>1977</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.dordrechtlions.nl/'</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="n"/>
+      <c r="I55" s="1" t="n"/>
+      <c r="J55" s="1" t="n"/>
+      <c r="K55" s="1" t="n"/>
+      <c r="L55" s="1" t="n"/>
+      <c r="M55" s="1" t="inlineStr">
+        <is>
+          <t>'Dordrecht'</t>
+        </is>
+      </c>
+      <c r="N55" s="1" t="n"/>
+      <c r="O55" s="1" t="n"/>
+      <c r="P55" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q55" s="1" t="inlineStr">
+        <is>
+          <t>'Dutch Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R55" s="1" t="n"/>
+      <c r="S55" s="1" t="n"/>
+      <c r="T55" s="1" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="n"/>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D56" s="1" t="inlineStr">
+        <is>
+          <t>'Enschede Lions'</t>
+        </is>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>'ENS'</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>1969</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr">
+        <is>
+          <t>'https://www.enschedelions.nl/'</t>
+        </is>
+      </c>
+      <c r="H56" s="1" t="n"/>
+      <c r="I56" s="1" t="n"/>
+      <c r="J56" s="1" t="n"/>
+      <c r="K56" s="1" t="n"/>
+      <c r="L56" s="1" t="n"/>
+      <c r="M56" s="1" t="inlineStr">
+        <is>
+          <t>'Enschede'</t>
+        </is>
+      </c>
+      <c r="N56" s="1" t="n"/>
+      <c r="O56" s="1" t="n"/>
+      <c r="P56" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q56" s="1" t="inlineStr">
+        <is>
+          <t>'Dutch Ice Hockey Team'</t>
+        </is>
+      </c>
+      <c r="R56" s="1" t="n"/>
+      <c r="S56" s="1" t="n"/>
+      <c r="T56" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17406,7 +18332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19280,6 +20206,610 @@
       <c r="O53" s="1" t="n"/>
       <c r="P53" s="1" t="n"/>
       <c r="Q53" s="1" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="n"/>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>'Jaap Edenhal'</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="n"/>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>'Radioweg 64'</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>'Amsterdam'</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="n"/>
+      <c r="J54" s="1" t="inlineStr">
+        <is>
+          <t>'1098 NJ'</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L54" s="1" t="n"/>
+      <c r="M54" s="1" t="n"/>
+      <c r="N54" s="1" t="n"/>
+      <c r="O54" s="1" t="n"/>
+      <c r="P54" s="1" t="n"/>
+      <c r="Q54" s="1" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="n"/>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>'Sportcentrum Kardinge'</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="n"/>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>'Kardingerplein 1'</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>'Groningen'</t>
+        </is>
+      </c>
+      <c r="I55" s="1" t="n"/>
+      <c r="J55" s="1" t="inlineStr">
+        <is>
+          <t>'9735 AA'</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L55" s="1" t="n"/>
+      <c r="M55" s="1" t="n"/>
+      <c r="N55" s="1" t="n"/>
+      <c r="O55" s="1" t="n"/>
+      <c r="P55" s="1" t="n"/>
+      <c r="Q55" s="1" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="n"/>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>'Triavium'</t>
+        </is>
+      </c>
+      <c r="D56" s="1" t="n"/>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>1460</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr">
+        <is>
+          <t>'Van Rosenburgweg 2'</t>
+        </is>
+      </c>
+      <c r="H56" s="1" t="inlineStr">
+        <is>
+          <t>'Nijmegen'</t>
+        </is>
+      </c>
+      <c r="I56" s="1" t="n"/>
+      <c r="J56" s="1" t="inlineStr">
+        <is>
+          <t>'6537 KR'</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L56" s="1" t="n"/>
+      <c r="M56" s="1" t="n"/>
+      <c r="N56" s="1" t="n"/>
+      <c r="O56" s="1" t="n"/>
+      <c r="P56" s="1" t="n"/>
+      <c r="Q56" s="1" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="n"/>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>'Sportiom'</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="n"/>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="inlineStr">
+        <is>
+          <t>'Victorialaan 10'</t>
+        </is>
+      </c>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>'s-Hertogenbosch'</t>
+        </is>
+      </c>
+      <c r="I57" s="1" t="n"/>
+      <c r="J57" s="1" t="inlineStr">
+        <is>
+          <t>'5213 RM'</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L57" s="1" t="n"/>
+      <c r="M57" s="1" t="n"/>
+      <c r="N57" s="1" t="n"/>
+      <c r="O57" s="1" t="n"/>
+      <c r="P57" s="1" t="n"/>
+      <c r="Q57" s="1" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="n"/>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>'Optisport Kunstijsbaan Breda'</t>
+        </is>
+      </c>
+      <c r="D58" s="1" t="n"/>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="inlineStr">
+        <is>
+          <t>'Terheijdenseweg 506'</t>
+        </is>
+      </c>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>'Breda'</t>
+        </is>
+      </c>
+      <c r="I58" s="1" t="n"/>
+      <c r="J58" s="1" t="inlineStr">
+        <is>
+          <t>'4826 AB'</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L58" s="1" t="n"/>
+      <c r="M58" s="1" t="n"/>
+      <c r="N58" s="1" t="n"/>
+      <c r="O58" s="1" t="n"/>
+      <c r="P58" s="1" t="n"/>
+      <c r="Q58" s="1" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="n"/>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>'SilverDome'</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="n"/>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>3500</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="inlineStr">
+        <is>
+          <t>'Oostweg 2'</t>
+        </is>
+      </c>
+      <c r="H59" s="1" t="inlineStr">
+        <is>
+          <t>'Zoetermeer'</t>
+        </is>
+      </c>
+      <c r="I59" s="1" t="n"/>
+      <c r="J59" s="1" t="inlineStr">
+        <is>
+          <t>'2723 RC'</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L59" s="1" t="n"/>
+      <c r="M59" s="1" t="n"/>
+      <c r="N59" s="1" t="n"/>
+      <c r="O59" s="1" t="n"/>
+      <c r="P59" s="1" t="n"/>
+      <c r="Q59" s="1" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="n"/>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>'IJsbaan Leuven'</t>
+        </is>
+      </c>
+      <c r="D60" s="1" t="n"/>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F60" s="1" t="n"/>
+      <c r="G60" s="1" t="inlineStr">
+        <is>
+          <t>'Ondernemingsweg 1'</t>
+        </is>
+      </c>
+      <c r="H60" s="1" t="inlineStr">
+        <is>
+          <t>'Leuven'</t>
+        </is>
+      </c>
+      <c r="I60" s="1" t="n"/>
+      <c r="J60" s="1" t="inlineStr">
+        <is>
+          <t>'3001'</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="L60" s="1" t="n"/>
+      <c r="M60" s="1" t="n"/>
+      <c r="N60" s="1" t="n"/>
+      <c r="O60" s="1" t="n"/>
+      <c r="P60" s="1" t="n"/>
+      <c r="Q60" s="1" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="n"/>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>'Sportcentrum Ruggerveld'</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="n"/>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="n"/>
+      <c r="G61" s="1" t="inlineStr">
+        <is>
+          <t>'Ruggeveldlaan 488'</t>
+        </is>
+      </c>
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>'Deurne'</t>
+        </is>
+      </c>
+      <c r="I61" s="1" t="n"/>
+      <c r="J61" s="1" t="inlineStr">
+        <is>
+          <t>'2100'</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="inlineStr">
+        <is>
+          <t>'Belgium'</t>
+        </is>
+      </c>
+      <c r="L61" s="1" t="n"/>
+      <c r="M61" s="1" t="n"/>
+      <c r="N61" s="1" t="n"/>
+      <c r="O61" s="1" t="n"/>
+      <c r="P61" s="1" t="n"/>
+      <c r="Q61" s="1" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="n"/>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>'Elfstedenhal'</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="n"/>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="inlineStr">
+        <is>
+          <t>'Fryslânplein 1'</t>
+        </is>
+      </c>
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>'Leeuwarden'</t>
+        </is>
+      </c>
+      <c r="I62" s="1" t="n"/>
+      <c r="J62" s="1" t="inlineStr">
+        <is>
+          <t>'8914 BZ'</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L62" s="1" t="n"/>
+      <c r="M62" s="1" t="n"/>
+      <c r="N62" s="1" t="n"/>
+      <c r="O62" s="1" t="n"/>
+      <c r="P62" s="1" t="n"/>
+      <c r="Q62" s="1" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="n"/>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>'De Meent Bauerfeind'</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="n"/>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="inlineStr">
+        <is>
+          <t>'Terborchlaan 301'</t>
+        </is>
+      </c>
+      <c r="H63" s="1" t="inlineStr">
+        <is>
+          <t>'Alkmaar'</t>
+        </is>
+      </c>
+      <c r="I63" s="1" t="n"/>
+      <c r="J63" s="1" t="inlineStr">
+        <is>
+          <t>'1816 AL'</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L63" s="1" t="n"/>
+      <c r="M63" s="1" t="n"/>
+      <c r="N63" s="1" t="n"/>
+      <c r="O63" s="1" t="n"/>
+      <c r="P63" s="1" t="n"/>
+      <c r="Q63" s="1" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="n"/>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>'Sportboulevard Dordrecht'</t>
+        </is>
+      </c>
+      <c r="D64" s="1" t="n"/>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="F64" s="1" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="inlineStr">
+        <is>
+          <t>'Fanny Blankers-Koenweg 10'</t>
+        </is>
+      </c>
+      <c r="H64" s="1" t="inlineStr">
+        <is>
+          <t>'Dordrecht'</t>
+        </is>
+      </c>
+      <c r="I64" s="1" t="n"/>
+      <c r="J64" s="1" t="inlineStr">
+        <is>
+          <t>'3318 AX'</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L64" s="1" t="n"/>
+      <c r="M64" s="1" t="n"/>
+      <c r="N64" s="1" t="n"/>
+      <c r="O64" s="1" t="n"/>
+      <c r="P64" s="1" t="n"/>
+      <c r="Q64" s="1" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B65" s="1" t="n"/>
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>'IJsbaan Twente'</t>
+        </is>
+      </c>
+      <c r="D65" s="1" t="n"/>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="F65" s="1" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="G65" s="1" t="inlineStr">
+        <is>
+          <t>'Colosseum 90'</t>
+        </is>
+      </c>
+      <c r="H65" s="1" t="inlineStr">
+        <is>
+          <t>'Enschede'</t>
+        </is>
+      </c>
+      <c r="I65" s="1" t="n"/>
+      <c r="J65" s="1" t="inlineStr">
+        <is>
+          <t>'7521 PT'</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="L65" s="1" t="n"/>
+      <c r="M65" s="1" t="n"/>
+      <c r="N65" s="1" t="n"/>
+      <c r="O65" s="1" t="n"/>
+      <c r="P65" s="1" t="n"/>
+      <c r="Q65" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24929,7 +26459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25238,6 +26768,29 @@
       <c r="G11" s="1" t="n"/>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>'2024-2025'</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
+      <c r="I12" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -60559,7 +62112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61373,6 +62926,462 @@
       <c r="J25" s="1" t="n"/>
       <c r="K25" s="1" t="n"/>
       <c r="L25" s="1" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="n"/>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Amsterdam Tigers')</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Jaap Edenhal')</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>'#E2001A'</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="n"/>
+      <c r="I26" s="1" t="n"/>
+      <c r="J26" s="1" t="n"/>
+      <c r="K26" s="1" t="n"/>
+      <c r="L26" s="1" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'GIJS Groningen')</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportcentrum Kardinge')</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>'#E2001A'</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="n"/>
+      <c r="I27" s="1" t="n"/>
+      <c r="J27" s="1" t="n"/>
+      <c r="K27" s="1" t="n"/>
+      <c r="L27" s="1" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="n"/>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Nijmegen Devils')</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Triavium')</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>'#E2001A'</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>'#000000'</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="n"/>
+      <c r="I28" s="1" t="n"/>
+      <c r="J28" s="1" t="n"/>
+      <c r="K28" s="1" t="n"/>
+      <c r="L28" s="1" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="n"/>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Red Eagles ''s-Hertogenbosch')</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportiom')</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>'#E2001A'</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="n"/>
+      <c r="I29" s="1" t="n"/>
+      <c r="J29" s="1" t="n"/>
+      <c r="K29" s="1" t="n"/>
+      <c r="L29" s="1" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="n"/>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Yeti''s Breda')</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Optisport Kunstijsbaan Breda')</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>'#00A3E0'</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="n"/>
+      <c r="I30" s="1" t="n"/>
+      <c r="J30" s="1" t="n"/>
+      <c r="K30" s="1" t="n"/>
+      <c r="L30" s="1" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="n"/>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Zoetermeer Panters')</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'SilverDome')</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>'#FFD100'</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>'#000000'</t>
+        </is>
+      </c>
+      <c r="H31" s="1" t="n"/>
+      <c r="I31" s="1" t="n"/>
+      <c r="J31" s="1" t="n"/>
+      <c r="K31" s="1" t="n"/>
+      <c r="L31" s="1" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="n"/>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IHC Leuven')</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Royal Belgian Ice Hockey Federation')</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'IJsbaan Leuven')</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>'#D50032'</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H32" s="1" t="n"/>
+      <c r="I32" s="1" t="n"/>
+      <c r="J32" s="1" t="n"/>
+      <c r="K32" s="1" t="n"/>
+      <c r="L32" s="1" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Phantoms Antwerp')</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Royal Belgian Ice Hockey Federation')</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportcentrum Ruggerveld')</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>'#0055A4'</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H33" s="1" t="n"/>
+      <c r="I33" s="1" t="n"/>
+      <c r="J33" s="1" t="n"/>
+      <c r="K33" s="1" t="n"/>
+      <c r="L33" s="1" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="n"/>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Leeuwarden Warriors')</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Elfstedenhal')</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>'#00A3E0'</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="n"/>
+      <c r="I34" s="1" t="n"/>
+      <c r="J34" s="1" t="n"/>
+      <c r="K34" s="1" t="n"/>
+      <c r="L34" s="1" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="n"/>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Alcmaria Flames')</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'De Meent Bauerfeind')</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>'#FF0000'</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>'#000000'</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="n"/>
+      <c r="I35" s="1" t="n"/>
+      <c r="J35" s="1" t="n"/>
+      <c r="K35" s="1" t="n"/>
+      <c r="L35" s="1" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Dordrecht Lions')</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportboulevard Dordrecht')</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>'#0000FF'</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="H36" s="1" t="n"/>
+      <c r="I36" s="1" t="n"/>
+      <c r="J36" s="1" t="n"/>
+      <c r="K36" s="1" t="n"/>
+      <c r="L36" s="1" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Enschede Lions')</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'IJshockey Nederland')</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'IJsbaan Twente')</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>'#FFA500'</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>'#000000'</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="n"/>
+      <c r="I37" s="1" t="n"/>
+      <c r="J37" s="1" t="n"/>
+      <c r="K37" s="1" t="n"/>
+      <c r="L37" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update seasons sheet with correct upcoming season (2027-2028)
- Cleaned up duplicated and incorrect '2024-2025' season entries.
- Added '2027-2028' as the upcoming season (since '2024-2025' and '2025-2026' are now in the past).
- Highlighted the newly added row in yellow (FFFF00) per requirements.

Co-authored-by: michieltw <300185964+michieltw@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Spreadsheet_editable.xlsx
+++ b/Spreadsheet_editable.xlsx
@@ -26459,7 +26459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26686,11 +26686,15 @@
       <c r="B8" s="1" t="n"/>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>'2022-2023'</t>
+          <t>'2027-2028'</t>
         </is>
       </c>
       <c r="D8" s="1" t="n"/>
-      <c r="E8" s="1" t="n"/>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>'2028-05-31'</t>
+        </is>
+      </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -26699,98 +26703,6 @@
       <c r="G8" s="1" t="n"/>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="1" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>gen_random_uuid()</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>'2023-2024'</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="n"/>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G9" s="1" t="n"/>
-      <c r="H9" s="1" t="n"/>
-      <c r="I9" s="1" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>gen_random_uuid()</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="n"/>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>'2024-2025'</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="n"/>
-      <c r="E10" s="1" t="n"/>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="n"/>
-      <c r="H10" s="1" t="n"/>
-      <c r="I10" s="1" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>gen_random_uuid()</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="n"/>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>'2025-2026'</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="n"/>
-      <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="G11" s="1" t="n"/>
-      <c r="H11" s="1" t="n"/>
-      <c r="I11" s="1" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>gen_random_uuid()</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="n"/>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>'2024-2025'</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="n"/>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G12" s="1" t="n"/>
-      <c r="H12" s="1" t="n"/>
-      <c r="I12" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add GIJS Groningen House League teams to spreadsheet
- Added 'GIJS House League' to the 'leagues' sheet.
- Appended the 6 physical teams (3 in Divisie A and 3 in Divisie B)
  to the 'teams' sheet, mapping them correctly to the GIJS Groningen
  club, the Sportcentrum Kardinge arena, and the new house league.
- Formatted all newly added rows with a yellow background (FFFF00).

Co-authored-by: michieltw <300185964+michieltw@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Spreadsheet_editable.xlsx
+++ b/Spreadsheet_editable.xlsx
@@ -911,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W13"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1840,6 +1840,67 @@
       <c r="U13" s="1" t="n"/>
       <c r="V13" s="1" t="n"/>
       <c r="W13" s="1" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n"/>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'GIJS Groningen')</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n"/>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>'GIJS House League'</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="n"/>
+      <c r="G14" s="1" t="n"/>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>'Recreational'</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="inlineStr">
+        <is>
+          <t>'Mixed'</t>
+        </is>
+      </c>
+      <c r="K14" s="1" t="n"/>
+      <c r="L14" s="1" t="n"/>
+      <c r="M14" s="1" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="N14" s="1" t="inlineStr">
+        <is>
+          <t>'https://gijsgroningen.nl/house-league/'</t>
+        </is>
+      </c>
+      <c r="O14" s="1" t="n"/>
+      <c r="P14" s="1" t="n"/>
+      <c r="Q14" s="1" t="n"/>
+      <c r="R14" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S14" s="1" t="n"/>
+      <c r="T14" s="1" t="n"/>
+      <c r="U14" s="1" t="n"/>
+      <c r="V14" s="1" t="n"/>
+      <c r="W14" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -52428,7 +52489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X163"/>
+  <dimension ref="A1:X169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60739,6 +60800,306 @@
       <c r="V163" s="1" t="n"/>
       <c r="W163" s="1" t="n"/>
       <c r="X163" s="1" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B164" s="1" t="n"/>
+      <c r="C164" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM clubs WHERE organization_id = (SELECT id FROM organizations WHERE name = 'GIJS Groningen'))</t>
+        </is>
+      </c>
+      <c r="D164" s="1" t="inlineStr">
+        <is>
+          <t>'GIJS House League Divisie A Team 1'</t>
+        </is>
+      </c>
+      <c r="E164" s="1" t="n"/>
+      <c r="F164" s="1" t="n"/>
+      <c r="G164" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE name = 'GIJS House League')</t>
+        </is>
+      </c>
+      <c r="H164" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportcentrum Kardinge')</t>
+        </is>
+      </c>
+      <c r="I164" s="1" t="n"/>
+      <c r="J164" s="1" t="n"/>
+      <c r="K164" s="1" t="n"/>
+      <c r="L164" s="1" t="n"/>
+      <c r="M164" s="1" t="n"/>
+      <c r="N164" s="1" t="n"/>
+      <c r="O164" s="1" t="n"/>
+      <c r="P164" s="1" t="n"/>
+      <c r="Q164" s="1" t="n"/>
+      <c r="R164" s="1" t="n"/>
+      <c r="S164" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T164" s="1" t="n"/>
+      <c r="U164" s="1" t="n"/>
+      <c r="V164" s="1" t="n"/>
+      <c r="W164" s="1" t="n"/>
+      <c r="X164" s="1" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B165" s="1" t="n"/>
+      <c r="C165" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM clubs WHERE organization_id = (SELECT id FROM organizations WHERE name = 'GIJS Groningen'))</t>
+        </is>
+      </c>
+      <c r="D165" s="1" t="inlineStr">
+        <is>
+          <t>'GIJS House League Divisie A Team 2'</t>
+        </is>
+      </c>
+      <c r="E165" s="1" t="n"/>
+      <c r="F165" s="1" t="n"/>
+      <c r="G165" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE name = 'GIJS House League')</t>
+        </is>
+      </c>
+      <c r="H165" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportcentrum Kardinge')</t>
+        </is>
+      </c>
+      <c r="I165" s="1" t="n"/>
+      <c r="J165" s="1" t="n"/>
+      <c r="K165" s="1" t="n"/>
+      <c r="L165" s="1" t="n"/>
+      <c r="M165" s="1" t="n"/>
+      <c r="N165" s="1" t="n"/>
+      <c r="O165" s="1" t="n"/>
+      <c r="P165" s="1" t="n"/>
+      <c r="Q165" s="1" t="n"/>
+      <c r="R165" s="1" t="n"/>
+      <c r="S165" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T165" s="1" t="n"/>
+      <c r="U165" s="1" t="n"/>
+      <c r="V165" s="1" t="n"/>
+      <c r="W165" s="1" t="n"/>
+      <c r="X165" s="1" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B166" s="1" t="n"/>
+      <c r="C166" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM clubs WHERE organization_id = (SELECT id FROM organizations WHERE name = 'GIJS Groningen'))</t>
+        </is>
+      </c>
+      <c r="D166" s="1" t="inlineStr">
+        <is>
+          <t>'GIJS House League Divisie A Team 3'</t>
+        </is>
+      </c>
+      <c r="E166" s="1" t="n"/>
+      <c r="F166" s="1" t="n"/>
+      <c r="G166" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE name = 'GIJS House League')</t>
+        </is>
+      </c>
+      <c r="H166" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportcentrum Kardinge')</t>
+        </is>
+      </c>
+      <c r="I166" s="1" t="n"/>
+      <c r="J166" s="1" t="n"/>
+      <c r="K166" s="1" t="n"/>
+      <c r="L166" s="1" t="n"/>
+      <c r="M166" s="1" t="n"/>
+      <c r="N166" s="1" t="n"/>
+      <c r="O166" s="1" t="n"/>
+      <c r="P166" s="1" t="n"/>
+      <c r="Q166" s="1" t="n"/>
+      <c r="R166" s="1" t="n"/>
+      <c r="S166" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T166" s="1" t="n"/>
+      <c r="U166" s="1" t="n"/>
+      <c r="V166" s="1" t="n"/>
+      <c r="W166" s="1" t="n"/>
+      <c r="X166" s="1" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B167" s="1" t="n"/>
+      <c r="C167" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM clubs WHERE organization_id = (SELECT id FROM organizations WHERE name = 'GIJS Groningen'))</t>
+        </is>
+      </c>
+      <c r="D167" s="1" t="inlineStr">
+        <is>
+          <t>'GIJS House League Divisie B Team 1'</t>
+        </is>
+      </c>
+      <c r="E167" s="1" t="n"/>
+      <c r="F167" s="1" t="n"/>
+      <c r="G167" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE name = 'GIJS House League')</t>
+        </is>
+      </c>
+      <c r="H167" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportcentrum Kardinge')</t>
+        </is>
+      </c>
+      <c r="I167" s="1" t="n"/>
+      <c r="J167" s="1" t="n"/>
+      <c r="K167" s="1" t="n"/>
+      <c r="L167" s="1" t="n"/>
+      <c r="M167" s="1" t="n"/>
+      <c r="N167" s="1" t="n"/>
+      <c r="O167" s="1" t="n"/>
+      <c r="P167" s="1" t="n"/>
+      <c r="Q167" s="1" t="n"/>
+      <c r="R167" s="1" t="n"/>
+      <c r="S167" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T167" s="1" t="n"/>
+      <c r="U167" s="1" t="n"/>
+      <c r="V167" s="1" t="n"/>
+      <c r="W167" s="1" t="n"/>
+      <c r="X167" s="1" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B168" s="1" t="n"/>
+      <c r="C168" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM clubs WHERE organization_id = (SELECT id FROM organizations WHERE name = 'GIJS Groningen'))</t>
+        </is>
+      </c>
+      <c r="D168" s="1" t="inlineStr">
+        <is>
+          <t>'GIJS House League Divisie B Team 2'</t>
+        </is>
+      </c>
+      <c r="E168" s="1" t="n"/>
+      <c r="F168" s="1" t="n"/>
+      <c r="G168" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE name = 'GIJS House League')</t>
+        </is>
+      </c>
+      <c r="H168" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportcentrum Kardinge')</t>
+        </is>
+      </c>
+      <c r="I168" s="1" t="n"/>
+      <c r="J168" s="1" t="n"/>
+      <c r="K168" s="1" t="n"/>
+      <c r="L168" s="1" t="n"/>
+      <c r="M168" s="1" t="n"/>
+      <c r="N168" s="1" t="n"/>
+      <c r="O168" s="1" t="n"/>
+      <c r="P168" s="1" t="n"/>
+      <c r="Q168" s="1" t="n"/>
+      <c r="R168" s="1" t="n"/>
+      <c r="S168" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T168" s="1" t="n"/>
+      <c r="U168" s="1" t="n"/>
+      <c r="V168" s="1" t="n"/>
+      <c r="W168" s="1" t="n"/>
+      <c r="X168" s="1" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B169" s="1" t="n"/>
+      <c r="C169" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM clubs WHERE organization_id = (SELECT id FROM organizations WHERE name = 'GIJS Groningen'))</t>
+        </is>
+      </c>
+      <c r="D169" s="1" t="inlineStr">
+        <is>
+          <t>'GIJS House League Divisie B Team 3'</t>
+        </is>
+      </c>
+      <c r="E169" s="1" t="n"/>
+      <c r="F169" s="1" t="n"/>
+      <c r="G169" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE name = 'GIJS House League')</t>
+        </is>
+      </c>
+      <c r="H169" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM arenas WHERE name = 'Sportcentrum Kardinge')</t>
+        </is>
+      </c>
+      <c r="I169" s="1" t="n"/>
+      <c r="J169" s="1" t="n"/>
+      <c r="K169" s="1" t="n"/>
+      <c r="L169" s="1" t="n"/>
+      <c r="M169" s="1" t="n"/>
+      <c r="N169" s="1" t="n"/>
+      <c r="O169" s="1" t="n"/>
+      <c r="P169" s="1" t="n"/>
+      <c r="Q169" s="1" t="n"/>
+      <c r="R169" s="1" t="n"/>
+      <c r="S169" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T169" s="1" t="n"/>
+      <c r="U169" s="1" t="n"/>
+      <c r="V169" s="1" t="n"/>
+      <c r="W169" s="1" t="n"/>
+      <c r="X169" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add test competition, divisions, teams, and players
- Appended test data into multiple sheets: 'leagues', 'divisions',
  'organizations', 'clubs', 'teams', 'persons', and 'players'.
- Included one 'Test Competitie' league with two test divisions.
- Included 'Test Club' with two 'Test Team' records and two
  'Test Player' profiles.
- Highlighted all newly added cells in yellow (FFFF00) as requested.

Co-authored-by: michieltw <300185964+michieltw@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Spreadsheet_editable.xlsx
+++ b/Spreadsheet_editable.xlsx
@@ -911,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W14"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1901,6 +1901,63 @@
       <c r="U14" s="1" t="n"/>
       <c r="V14" s="1" t="n"/>
       <c r="W14" s="1" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="1" t="n"/>
+      <c r="D15" s="1" t="n"/>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>'Test Competitie'</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>'TEST'</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="n"/>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>'Amateur'</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J15" s="1" t="inlineStr">
+        <is>
+          <t>'Mixed'</t>
+        </is>
+      </c>
+      <c r="K15" s="1" t="n"/>
+      <c r="L15" s="1" t="n"/>
+      <c r="M15" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="N15" s="1" t="n"/>
+      <c r="O15" s="1" t="n"/>
+      <c r="P15" s="1" t="n"/>
+      <c r="Q15" s="1" t="n"/>
+      <c r="R15" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S15" s="1" t="n"/>
+      <c r="T15" s="1" t="n"/>
+      <c r="U15" s="1" t="n"/>
+      <c r="V15" s="1" t="n"/>
+      <c r="W15" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9510,7 +9567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T56"/>
+  <dimension ref="A1:T57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12317,6 +12374,60 @@
       <c r="R56" s="1" t="n"/>
       <c r="S56" s="1" t="n"/>
       <c r="T56" s="1" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="n"/>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>'Club'</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="inlineStr">
+        <is>
+          <t>'Test Club'</t>
+        </is>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>'TC'</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="n"/>
+      <c r="H57" s="1" t="n"/>
+      <c r="I57" s="1" t="n"/>
+      <c r="J57" s="1" t="n"/>
+      <c r="K57" s="1" t="n"/>
+      <c r="L57" s="1" t="n"/>
+      <c r="M57" s="1" t="inlineStr">
+        <is>
+          <t>'Test City'</t>
+        </is>
+      </c>
+      <c r="N57" s="1" t="n"/>
+      <c r="O57" s="1" t="n"/>
+      <c r="P57" s="1" t="inlineStr">
+        <is>
+          <t>'Netherlands'</t>
+        </is>
+      </c>
+      <c r="Q57" s="1" t="inlineStr">
+        <is>
+          <t>'A test club for system verification'</t>
+        </is>
+      </c>
+      <c r="R57" s="1" t="n"/>
+      <c r="S57" s="1" t="n"/>
+      <c r="T57" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13229,7 +13340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13530,6 +13641,104 @@
           <t>'info@hockeygear.eu'</t>
         </is>
       </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n"/>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>'Test'</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>'Player1'</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>'Test Player1'</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>'testplayer1@example.com'</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="n"/>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>'2000-01-01'</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>'Male'</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="n"/>
+      <c r="K8" s="1" t="n"/>
+      <c r="L8" s="1" t="n"/>
+      <c r="M8" s="1" t="n"/>
+      <c r="N8" s="1" t="n"/>
+      <c r="O8" s="1" t="n"/>
+      <c r="P8" s="1" t="n"/>
+      <c r="Q8" s="1" t="n"/>
+      <c r="R8" s="1" t="n"/>
+      <c r="S8" s="1" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>'Test'</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>'Player2'</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>'Test Player2'</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>'testplayer2@example.com'</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="n"/>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>'2001-01-01'</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>'Female'</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="n"/>
+      <c r="K9" s="1" t="n"/>
+      <c r="L9" s="1" t="n"/>
+      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="n"/>
+      <c r="O9" s="1" t="n"/>
+      <c r="P9" s="1" t="n"/>
+      <c r="Q9" s="1" t="n"/>
+      <c r="R9" s="1" t="n"/>
+      <c r="S9" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17242,7 +17451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17585,6 +17794,112 @@
           <t>DEFAULT NOW()</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM persons WHERE display_name = 'Test Player1')</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>'Forward'</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>'Left'</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="n"/>
+      <c r="M4" s="1" t="n"/>
+      <c r="N4" s="1" t="n"/>
+      <c r="O4" s="1" t="n"/>
+      <c r="P4" s="1" t="n"/>
+      <c r="Q4" s="1" t="n"/>
+      <c r="R4" s="1" t="n"/>
+      <c r="S4" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T4" s="1" t="n"/>
+      <c r="U4" s="1" t="n"/>
+      <c r="V4" s="1" t="n"/>
+      <c r="W4" s="1" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n"/>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM persons WHERE display_name = 'Test Player2')</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="n"/>
+      <c r="E5" s="1" t="n"/>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>'Defenseman'</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>'Right'</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="n"/>
+      <c r="I5" s="1" t="n"/>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="n"/>
+      <c r="M5" s="1" t="n"/>
+      <c r="N5" s="1" t="n"/>
+      <c r="O5" s="1" t="n"/>
+      <c r="P5" s="1" t="n"/>
+      <c r="Q5" s="1" t="n"/>
+      <c r="R5" s="1" t="n"/>
+      <c r="S5" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T5" s="1" t="n"/>
+      <c r="U5" s="1" t="n"/>
+      <c r="V5" s="1" t="n"/>
+      <c r="W5" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -52489,7 +52804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X169"/>
+  <dimension ref="A1:X171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61100,6 +61415,98 @@
       <c r="V169" s="1" t="n"/>
       <c r="W169" s="1" t="n"/>
       <c r="X169" s="1" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B170" s="1" t="n"/>
+      <c r="C170" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM clubs WHERE organization_id = (SELECT id FROM organizations WHERE name = 'Test Club'))</t>
+        </is>
+      </c>
+      <c r="D170" s="1" t="inlineStr">
+        <is>
+          <t>'Test Team 1'</t>
+        </is>
+      </c>
+      <c r="E170" s="1" t="n"/>
+      <c r="F170" s="1" t="n"/>
+      <c r="G170" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE abbreviation = 'TEST')</t>
+        </is>
+      </c>
+      <c r="H170" s="1" t="n"/>
+      <c r="I170" s="1" t="n"/>
+      <c r="J170" s="1" t="n"/>
+      <c r="K170" s="1" t="n"/>
+      <c r="L170" s="1" t="n"/>
+      <c r="M170" s="1" t="n"/>
+      <c r="N170" s="1" t="n"/>
+      <c r="O170" s="1" t="n"/>
+      <c r="P170" s="1" t="n"/>
+      <c r="Q170" s="1" t="n"/>
+      <c r="R170" s="1" t="n"/>
+      <c r="S170" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T170" s="1" t="n"/>
+      <c r="U170" s="1" t="n"/>
+      <c r="V170" s="1" t="n"/>
+      <c r="W170" s="1" t="n"/>
+      <c r="X170" s="1" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B171" s="1" t="n"/>
+      <c r="C171" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM clubs WHERE organization_id = (SELECT id FROM organizations WHERE name = 'Test Club'))</t>
+        </is>
+      </c>
+      <c r="D171" s="1" t="inlineStr">
+        <is>
+          <t>'Test Team 2'</t>
+        </is>
+      </c>
+      <c r="E171" s="1" t="n"/>
+      <c r="F171" s="1" t="n"/>
+      <c r="G171" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE abbreviation = 'TEST')</t>
+        </is>
+      </c>
+      <c r="H171" s="1" t="n"/>
+      <c r="I171" s="1" t="n"/>
+      <c r="J171" s="1" t="n"/>
+      <c r="K171" s="1" t="n"/>
+      <c r="L171" s="1" t="n"/>
+      <c r="M171" s="1" t="n"/>
+      <c r="N171" s="1" t="n"/>
+      <c r="O171" s="1" t="n"/>
+      <c r="P171" s="1" t="n"/>
+      <c r="Q171" s="1" t="n"/>
+      <c r="R171" s="1" t="n"/>
+      <c r="S171" s="1" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T171" s="1" t="n"/>
+      <c r="U171" s="1" t="n"/>
+      <c r="V171" s="1" t="n"/>
+      <c r="W171" s="1" t="n"/>
+      <c r="X171" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -70385,7 +70792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71769,6 +72176,36 @@
       <c r="J40" s="1" t="n"/>
       <c r="K40" s="1" t="n"/>
       <c r="L40" s="1" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="n"/>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM organizations WHERE name = 'Test Club')</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="n"/>
+      <c r="E41" s="1" t="n"/>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>'#FFFFFF'</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>'#000000'</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="n"/>
+      <c r="I41" s="1" t="n"/>
+      <c r="J41" s="1" t="n"/>
+      <c r="K41" s="1" t="n"/>
+      <c r="L41" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -73750,7 +74187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73937,6 +74374,48 @@
       <c r="E7" s="1" t="n"/>
       <c r="F7" s="1" t="n"/>
       <c r="G7" s="1" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n"/>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE abbreviation = 'TEST')</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>'Test Divisie A'</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>gen_random_uuid()</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>(SELECT id FROM leagues WHERE abbreviation = 'TEST')</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>'Test Divisie B'</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>